<commit_message>
[Docs] Refresh benchmark reports with color metrics
</commit_message>
<xml_diff>
--- a/docs/image_benchmark/kodak/results.xlsx
+++ b/docs/image_benchmark/kodak/results.xlsx
@@ -12,9 +12,9 @@
     <sheet name="BD-Rate" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All metrics'!$A$1:$S$193</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Same-QP summary'!$A$1:$N$97</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BD-Rate'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All metrics'!$A$1:$U$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Same-QP summary'!$A$1:$P$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BD-Rate'!$A$1:$H$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S193"/>
+  <dimension ref="A1:U193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -459,6 +459,8 @@
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -557,6 +559,16 @@
           <t>psnr_hvs_m_luma</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>psnr_rgb</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>msssim_rgb</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -654,6 +666,16 @@
           <t>41.92482837549974</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>42.051972720159476</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>0.9994322624685138</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -751,6 +773,16 @@
           <t>40.975633302683924</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>41.397318617847986</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>0.9994171177127485</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -848,6 +880,16 @@
           <t>37.51317476951805</t>
         </is>
       </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>38.5528007201883</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>0.9987916753352808</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -945,6 +987,16 @@
           <t>36.62792905204792</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>37.85270753399511</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>0.998745078787255</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1042,6 +1094,16 @@
           <t>33.083198867916124</t>
         </is>
       </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>34.65756528111662</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>0.9973188483380043</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1139,6 +1201,16 @@
           <t>32.34559585205206</t>
         </is>
       </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>33.98482491681401</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>0.9971362754012015</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1236,6 +1308,16 @@
           <t>29.054981175950054</t>
         </is>
       </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>30.860127713628774</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>0.9935788461312742</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1333,6 +1415,16 @@
           <t>28.560221965751097</t>
         </is>
       </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>30.355787402898923</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>0.9930646020427597</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1430,6 +1522,16 @@
           <t>41.63536872878258</t>
         </is>
       </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>41.9415751852977</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>0.9985318370458763</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1527,6 +1629,16 @@
           <t>40.99287549808334</t>
         </is>
       </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>41.52129382550676</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>0.9984557766011378</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1624,6 +1736,16 @@
           <t>37.91235842257574</t>
         </is>
       </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>38.80843729202584</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>0.9967857719282479</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1721,6 +1843,16 @@
           <t>37.445404533360986</t>
         </is>
       </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>38.44935676373172</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>0.99666861939934</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1818,6 +1950,16 @@
           <t>34.56577615745882</t>
         </is>
       </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>35.83021080897372</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>0.9931450925672038</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1915,6 +2057,16 @@
           <t>34.27066254147992</t>
         </is>
       </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>35.61129489562444</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>0.9930519310653589</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2012,6 +2164,16 @@
           <t>31.820136932169728</t>
         </is>
       </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>33.22666619324624</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>0.9862285349303277</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2109,6 +2271,16 @@
           <t>31.689629924420878</t>
         </is>
       </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>33.08694537606017</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>0.9861478059579122</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2206,6 +2378,16 @@
           <t>43.16461447906116</t>
         </is>
       </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>43.57091159224833</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>0.9997157910352644</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2303,6 +2485,16 @@
           <t>42.77500524674459</t>
         </is>
       </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>43.31976965630173</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>0.9997100212538395</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2400,6 +2592,16 @@
           <t>40.19730056736876</t>
         </is>
       </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>41.04757208220381</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>0.9994329470294755</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2497,6 +2699,16 @@
           <t>39.84651940673047</t>
         </is>
       </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>40.79828030445746</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>0.9994138614813955</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2594,6 +2806,16 @@
           <t>37.09624519434178</t>
         </is>
       </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>38.25885301711728</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>0.9988245315858651</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2691,6 +2913,16 @@
           <t>36.729806281097964</t>
         </is>
       </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>37.99469153486073</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>0.9988134369004241</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2788,6 +3020,16 @@
           <t>33.94009075652755</t>
         </is>
       </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>35.33112475935953</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>0.9975486758968888</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2885,6 +3127,16 @@
           <t>33.65447262300032</t>
         </is>
       </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>35.17052708921954</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>0.9975727025310593</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2982,6 +3234,16 @@
           <t>41.73904804970776</t>
         </is>
       </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>42.184547845762324</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>0.9995249624946774</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3079,6 +3341,16 @@
           <t>41.02160403170249</t>
         </is>
       </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>41.69896759113143</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>0.9994962508074557</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3176,6 +3448,16 @@
           <t>38.11774867539154</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>39.12584635503263</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>0.9989535025150192</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3273,6 +3555,16 @@
           <t>37.4404867218296</t>
         </is>
       </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>38.63485430778653</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>0.9988947970553514</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3370,6 +3662,16 @@
           <t>34.763969719455595</t>
         </is>
       </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>36.16457812549002</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>0.9977849576027582</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3467,6 +3769,16 @@
           <t>34.228421615477245</t>
         </is>
       </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>35.71301713511119</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>0.9976606634992331</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3564,6 +3876,16 @@
           <t>31.87192115770404</t>
         </is>
       </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>33.312940107976786</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>0.9951568464465317</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3661,6 +3983,16 @@
           <t>31.61840723902999</t>
         </is>
       </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>33.11759954919958</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>0.995087172532593</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3758,6 +4090,16 @@
           <t>42.48628387689956</t>
         </is>
       </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>41.446978260145</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>0.9994845039955612</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3855,6 +4197,16 @@
           <t>41.748180871306076</t>
         </is>
       </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>40.995074440280355</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>0.999462979378657</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3952,6 +4304,16 @@
           <t>38.374153224253305</t>
         </is>
       </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>37.921391983702165</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>0.9987686449014577</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4049,6 +4411,16 @@
           <t>37.8013771561374</t>
         </is>
       </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>37.52688004868339</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>0.9987358907571625</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4146,6 +4518,16 @@
           <t>34.28312349063715</t>
         </is>
       </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>34.410029490674304</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>0.9972369084842724</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4243,6 +4625,16 @@
           <t>33.70842133063555</t>
         </is>
       </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>34.02252411593505</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>0.9971550432696548</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4340,6 +4732,16 @@
           <t>30.320712028769346</t>
         </is>
       </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>30.820335917136624</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>0.9935159386149174</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4437,6 +4839,16 @@
           <t>30.053877491525025</t>
         </is>
       </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>30.61771422367555</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>0.9934766088832472</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4534,6 +4946,16 @@
           <t>41.91325614816809</t>
         </is>
       </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>42.199717104199735</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>0.9997512520361362</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4631,6 +5053,16 @@
           <t>41.18834463337503</t>
         </is>
       </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>41.69727592995294</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>0.99974191049869</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4728,6 +5160,16 @@
           <t>37.98155338625916</t>
         </is>
       </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>39.00197915097956</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>0.99950190349171</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4825,6 +5267,16 @@
           <t>37.29433776055862</t>
         </is>
       </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>38.49448603596178</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>0.9994869157888816</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4922,6 +5374,16 @@
           <t>34.0839918019983</t>
         </is>
       </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>35.618387186733564</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>0.9989689762356724</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5019,6 +5481,16 @@
           <t>33.47865120855641</t>
         </is>
       </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>35.12180800636909</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>0.9989488973567427</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5116,6 +5588,16 @@
           <t>30.471072550224427</t>
         </is>
       </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>32.23116447912101</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>0.9977453748639039</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5213,6 +5695,16 @@
           <t>29.999165030157403</t>
         </is>
       </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>31.752070622845793</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>0.9976148566691179</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5310,6 +5802,16 @@
           <t>43.148871353624415</t>
         </is>
       </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>42.92664146684183</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>0.999563248465532</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5407,6 +5909,16 @@
           <t>42.837399786160475</t>
         </is>
       </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>42.71689511969848</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>0.9995541663148323</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5504,6 +6016,16 @@
           <t>40.38367434595224</t>
         </is>
       </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>40.21965482744093</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>0.9990195653503054</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5601,6 +6123,16 @@
           <t>40.09776964177781</t>
         </is>
       </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>40.017124737097745</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>0.9990055551777903</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5698,6 +6230,16 @@
           <t>37.26069128190127</t>
         </is>
       </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>37.31707349827891</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>0.9978617550257277</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5795,6 +6337,16 @@
           <t>37.01529601865461</t>
         </is>
       </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>37.172744390992925</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>0.9978554433939801</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5892,6 +6444,16 @@
           <t>33.94819335539814</t>
         </is>
       </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>34.149993334683614</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>0.9951413578798455</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5989,6 +6551,16 @@
           <t>33.77953824309208</t>
         </is>
       </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>34.0995158123034</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>0.9951807923122981</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6086,6 +6658,16 @@
           <t>42.02886469820851</t>
         </is>
       </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>41.215143098667454</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>0.999702281147727</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6183,6 +6765,16 @@
           <t>41.01402990957132</t>
         </is>
       </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>40.569185214049924</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>0.9996891100009204</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6280,6 +6872,16 @@
           <t>37.653569809955776</t>
         </is>
       </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>37.68022764703482</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>0.9993373327629665</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6377,6 +6979,16 @@
           <t>36.87501315541836</t>
         </is>
       </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>37.09762252198436</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>0.9993077669993027</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6474,6 +7086,16 @@
           <t>33.783588666438675</t>
         </is>
       </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>34.26516329099721</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>0.9985614491732954</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6571,6 +7193,16 @@
           <t>33.193343395495084</t>
         </is>
       </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>33.7838141464585</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>0.9985332460621473</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6668,6 +7300,16 @@
           <t>30.272834858112233</t>
         </is>
       </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>30.93333001993892</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>0.9968472359546438</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6765,6 +7407,16 @@
           <t>29.857094634169236</t>
         </is>
       </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>30.585735547274787</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>0.996786595858386</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6862,6 +7514,16 @@
           <t>40.807408500927835</t>
         </is>
       </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>41.91456470325093</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>0.9995043899912363</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6959,6 +7621,16 @@
           <t>40.41700723299768</t>
         </is>
       </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>41.656411957606224</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>0.9994883403992811</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7056,6 +7728,16 @@
           <t>38.861427197402705</t>
         </is>
       </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>40.03399654101007</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>0.9990970049345065</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7153,6 +7835,16 @@
           <t>38.582430076220305</t>
         </is>
       </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>39.823140433868915</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>0.9990874609699262</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7250,6 +7942,16 @@
           <t>36.53017877669937</t>
         </is>
       </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>37.80022176857424</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>0.9983042827711149</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7347,6 +8049,16 @@
           <t>36.20022041507524</t>
         </is>
       </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>37.551693389363656</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>0.998281767776481</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -7444,6 +8156,16 @@
           <t>33.78925500879642</t>
         </is>
       </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>35.141454391569134</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>0.9965186429577676</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7541,6 +8263,16 @@
           <t>33.55812177134321</t>
         </is>
       </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>34.92826029860141</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>0.9964814233096603</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7638,6 +8370,16 @@
           <t>41.13200736379731</t>
         </is>
       </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>42.05610702634498</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>0.9994996942277455</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7735,6 +8477,16 @@
           <t>40.64881968234012</t>
         </is>
       </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>41.72460459367318</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>0.9994818426090815</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7832,6 +8584,16 @@
           <t>38.708517797938725</t>
         </is>
       </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>39.77006379160565</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>0.9989968901937615</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7929,6 +8691,16 @@
           <t>38.453400903111145</t>
         </is>
       </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>39.57588601758852</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>0.9989857073718111</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8026,6 +8798,16 @@
           <t>36.12171618578128</t>
         </is>
       </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>37.34727852565483</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>0.9980050818891284</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8123,6 +8905,16 @@
           <t>35.92315653318239</t>
         </is>
       </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>37.19314780985437</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>0.9980014066287524</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -8220,6 +9012,16 @@
           <t>33.31932033256929</t>
         </is>
       </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>34.711874206545055</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>0.9959962141513247</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8317,6 +9119,16 @@
           <t>33.18128682156323</t>
         </is>
       </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>34.57590875668588</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>0.9960065699653767</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -8414,6 +9226,16 @@
           <t>42.07173921951181</t>
         </is>
       </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>42.129534696506006</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>0.9995391863356393</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8511,6 +9333,16 @@
           <t>41.27931185317095</t>
         </is>
       </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>41.64714170819408</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>0.9995230595620525</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8608,6 +9440,16 @@
           <t>38.058574743429354</t>
         </is>
       </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>38.83595784135791</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>0.9989794556862831</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -8705,6 +9547,16 @@
           <t>37.37092730471431</t>
         </is>
       </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>38.35337444613269</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>0.9989517862856326</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -8802,6 +9654,16 @@
           <t>34.308989123562014</t>
         </is>
       </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>35.5643681129644</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>0.9978678799874491</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8899,6 +9761,16 @@
           <t>33.843495490246845</t>
         </is>
       </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>35.206397176245</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>0.9978003961183979</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -8996,6 +9868,16 @@
           <t>30.94916667772707</t>
         </is>
       </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>32.41435877589561</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>0.9953911639678</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9093,6 +9975,16 @@
           <t>30.668393251102337</t>
         </is>
       </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>32.13841558271841</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>0.9951921681020224</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -9190,6 +10082,16 @@
           <t>41.74951385692645</t>
         </is>
       </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>42.54270735810165</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>0.9996916193662031</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9287,6 +10189,16 @@
           <t>41.141179503868585</t>
         </is>
       </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>42.117666266435585</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>0.9996817019426647</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -9384,6 +10296,16 @@
           <t>38.57983678144996</t>
         </is>
       </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>39.91291495379373</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>0.9993720543152392</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -9481,6 +10403,16 @@
           <t>38.106050049929536</t>
         </is>
       </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>39.546251622857746</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>0.9993509000711946</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9578,6 +10510,16 @@
           <t>35.50221184528614</t>
         </is>
       </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>37.12420486117069</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>0.9987000660466987</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9675,6 +10617,16 @@
           <t>35.12991004817947</t>
         </is>
       </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>36.85035416534359</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>0.9986695443296799</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -9772,6 +10724,16 @@
           <t>32.80635317481557</t>
         </is>
       </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>34.54716208149491</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>0.9973263140199814</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9869,6 +10831,16 @@
           <t>32.59915127687728</t>
         </is>
       </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>34.3717443543465</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>0.9973130351429659</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -9966,6 +10938,16 @@
           <t>42.004048495900015</t>
         </is>
       </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>41.10427712611505</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>0.9995879307457937</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -10063,6 +11045,16 @@
           <t>40.85660167369812</t>
         </is>
       </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>40.43653798037094</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>0.9995734827495962</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -10160,6 +11152,16 @@
           <t>37.26926367081764</t>
         </is>
       </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>37.39706573614745</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>0.9990699430353694</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10257,6 +11259,16 @@
           <t>36.237286337311716</t>
         </is>
       </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>36.66923550829569</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>0.9990316470105808</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -10354,6 +11366,16 @@
           <t>32.54759852861403</t>
         </is>
       </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>33.56337158086024</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>0.9980421402941092</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -10451,6 +11473,16 @@
           <t>31.58422753382463</t>
         </is>
       </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>32.75607504848048</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>0.9979216177504195</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -10548,6 +11580,16 @@
           <t>28.189698713245907</t>
         </is>
       </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>29.59971773467008</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>0.9954846985347775</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -10645,6 +11687,16 @@
           <t>27.58394937459112</t>
         </is>
       </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>29.04518371543283</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>0.9952852930798343</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -10742,6 +11794,16 @@
           <t>41.71134194437634</t>
         </is>
       </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>41.66150536796433</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>0.999555526447835</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -10839,6 +11901,16 @@
           <t>40.85068364006767</t>
         </is>
       </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>41.15805713599972</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>0.9995437875408241</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -10936,6 +12008,16 @@
           <t>37.48338487777366</t>
         </is>
       </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>38.10141002380577</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>0.9989853273189103</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -11033,6 +12115,16 @@
           <t>36.73051354580607</t>
         </is>
       </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>37.547445316664465</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>0.9989325893216262</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -11130,6 +12222,16 @@
           <t>33.43469594276528</t>
         </is>
       </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>34.56022742156798</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>0.9977771657322142</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -11227,6 +12329,16 @@
           <t>32.916484457622396</t>
         </is>
       </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>34.150064147460085</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>0.9976740304799798</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -11324,6 +12436,16 @@
           <t>29.855639316632168</t>
         </is>
       </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>31.122298548051354</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>0.9947961644445521</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -11421,6 +12543,16 @@
           <t>29.61295903661554</t>
         </is>
       </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>30.906036419997566</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>0.9946704526219422</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -11518,6 +12650,16 @@
           <t>42.23160315550243</t>
         </is>
       </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>42.456496726315684</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>0.9998680520347918</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -11615,6 +12757,16 @@
           <t>41.367132339055324</t>
         </is>
       </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>41.88473414078465</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>0.9998613310744101</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -11712,6 +12864,16 @@
           <t>38.749927856808625</t>
         </is>
       </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>39.47278522545436</t>
+        </is>
+      </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>0.9997372856471936</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -11809,6 +12971,16 @@
           <t>38.01604932121952</t>
         </is>
       </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>38.97327220570007</t>
+        </is>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>0.9997267793200306</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -11906,6 +13078,16 @@
           <t>35.47113539726819</t>
         </is>
       </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>36.61579794445429</t>
+        </is>
+      </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>0.9994909684718271</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -12003,6 +13185,16 @@
           <t>35.055553333690796</t>
         </is>
       </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>36.28377154297894</t>
+        </is>
+      </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>0.9994762998650142</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -12100,6 +13292,16 @@
           <t>32.60444082293613</t>
         </is>
       </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>33.78163991823722</t>
+        </is>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>0.9989378073101647</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -12197,6 +13399,16 @@
           <t>32.36932222582474</t>
         </is>
       </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>33.58036450254501</t>
+        </is>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>0.9989212689757361</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -12294,6 +13506,16 @@
           <t>42.04528573459018</t>
         </is>
       </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>42.82962236939348</t>
+        </is>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>0.9996515142282077</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -12391,6 +13613,16 @@
           <t>41.39286032267866</t>
         </is>
       </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>42.37369966728643</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>0.9996397285275083</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -12488,6 +13720,16 @@
           <t>38.37748789997559</t>
         </is>
       </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>39.94702963292089</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>0.9993269588454061</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -12585,6 +13827,16 @@
           <t>37.72333195919485</t>
         </is>
       </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>39.39594846772352</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>0.9992951057810497</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -12682,6 +13934,16 @@
           <t>34.74471218153814</t>
         </is>
       </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>36.75225059655438</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>0.9985997378921317</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -12779,6 +14041,16 @@
           <t>34.16380007882384</t>
         </is>
       </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>36.2511994996752</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>0.9985267130389269</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -12876,6 +14148,16 @@
           <t>31.457509581316444</t>
         </is>
       </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>33.66174867518053</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>0.9969728990231994</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -12973,6 +14255,16 @@
           <t>31.10812125691443</t>
         </is>
       </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>33.33884465243932</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>0.9968553520748866</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -13070,6 +14362,16 @@
           <t>41.7627637816077</t>
         </is>
       </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>42.331449803730024</t>
+        </is>
+      </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>0.9996733916218098</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -13167,6 +14469,16 @@
           <t>41.23534452456052</t>
         </is>
       </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>41.9684134753378</t>
+        </is>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>0.9996672377060963</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -13264,6 +14576,16 @@
           <t>38.62325877176049</t>
         </is>
       </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>39.6956915831722</t>
+        </is>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>0.9993820005560803</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -13361,6 +14683,16 @@
           <t>38.26723564439124</t>
         </is>
       </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>39.44011988821167</t>
+        </is>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>0.9993704542260894</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -13458,6 +14790,16 @@
           <t>35.45942912985264</t>
         </is>
       </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>36.9380962191354</t>
+        </is>
+      </c>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>0.998794727589178</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -13555,6 +14897,16 @@
           <t>35.26756990235153</t>
         </is>
       </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>36.75802573232429</t>
+        </is>
+      </c>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>0.9987662147375896</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -13652,6 +15004,16 @@
           <t>32.50504347352975</t>
         </is>
       </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>34.168543790986014</t>
+        </is>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>0.9975131353639889</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -13749,6 +15111,16 @@
           <t>32.375308638887844</t>
         </is>
       </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>34.06499912375516</t>
+        </is>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>0.9975021375266842</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -13846,6 +15218,16 @@
           <t>41.29595134766266</t>
         </is>
       </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>40.970588771981014</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>0.9990602815128381</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -13943,6 +15325,16 @@
           <t>40.098000313069534</t>
         </is>
       </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>40.25199520391321</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>0.999005134837824</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -14040,6 +15432,16 @@
           <t>37.20553223056819</t>
         </is>
       </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>37.456899993271044</t>
+        </is>
+      </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>0.9978041202732438</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -14137,6 +15539,16 @@
           <t>36.46520428281089</t>
         </is>
       </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>36.92969375720319</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>0.9976954056941892</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -14234,6 +15646,16 @@
           <t>33.67874444906383</t>
         </is>
       </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>34.401577397283916</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>0.9955876519753243</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -14331,6 +15753,16 @@
           <t>33.05981815927034</t>
         </is>
       </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>33.94352085893772</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>0.995404601458211</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -14428,6 +15860,16 @@
           <t>30.131240368035833</t>
         </is>
       </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>31.2242148037016</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>0.9908076815614774</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -14525,6 +15967,16 @@
           <t>29.657222723653625</t>
         </is>
       </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>30.82782076198161</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>0.9904913878940511</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -14622,6 +16074,16 @@
           <t>41.441501086427905</t>
         </is>
       </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>41.835532290155655</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>0.99963458916084</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -14719,6 +16181,16 @@
           <t>40.83298711800645</t>
         </is>
       </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>41.40887353763617</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>0.9996251973506691</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -14816,6 +16288,16 @@
           <t>38.07867678450921</t>
         </is>
       </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>39.116118548555846</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>0.9993127057404237</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -14913,6 +16395,16 @@
           <t>37.32566534716637</t>
         </is>
       </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>38.53630503448676</t>
+        </is>
+      </c>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>0.9992779377482027</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -15010,6 +16502,16 @@
           <t>34.4268011983539</t>
         </is>
       </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>36.01763889092823</t>
+        </is>
+      </c>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>0.9986413808012292</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -15107,6 +16609,16 @@
           <t>33.683671147425464</t>
         </is>
       </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>35.445488014164816</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>0.9985802255290507</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -15204,6 +16716,16 @@
           <t>31.036380494259692</t>
         </is>
       </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>32.88980032848039</t>
+        </is>
+      </c>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>0.9970916950660312</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -15301,6 +16823,16 @@
           <t>30.783482415931548</t>
         </is>
       </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>32.65574021160289</t>
+        </is>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>0.9970246728869167</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -15398,6 +16930,16 @@
           <t>42.865179772828895</t>
         </is>
       </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>42.646938898648656</t>
+        </is>
+      </c>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>0.9999056938588154</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -15495,6 +17037,16 @@
           <t>42.31596942614601</t>
         </is>
       </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>42.333889622853526</t>
+        </is>
+      </c>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>0.9999045382844026</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -15592,6 +17144,16 @@
           <t>39.85330224757463</t>
         </is>
       </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>40.250667249587366</t>
+        </is>
+      </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>0.9998357527611571</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -15689,6 +17251,16 @@
           <t>39.21499687497374</t>
         </is>
       </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>39.85998013675982</t>
+        </is>
+      </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>0.9998328724534108</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -15786,6 +17358,16 @@
           <t>36.34799697552093</t>
         </is>
       </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>37.3907365151275</t>
+        </is>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>0.9996975913355038</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -15883,6 +17465,16 @@
           <t>35.659028229722445</t>
         </is>
       </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>36.88265828774236</t>
+        </is>
+      </c>
+      <c r="U159" t="inlineStr">
+        <is>
+          <t>0.9996844541876464</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -15980,6 +17572,16 @@
           <t>33.03676933621636</t>
         </is>
       </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>34.36751636048108</t>
+        </is>
+      </c>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>0.9993621200710749</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -16077,6 +17679,16 @@
           <t>32.797106740306674</t>
         </is>
       </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t>34.197889459516176</t>
+        </is>
+      </c>
+      <c r="U161" t="inlineStr">
+        <is>
+          <t>0.9993556210235363</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -16174,6 +17786,16 @@
           <t>41.29559381708223</t>
         </is>
       </c>
+      <c r="T162" t="inlineStr">
+        <is>
+          <t>41.65120916184296</t>
+        </is>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>0.9995887996690304</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -16271,6 +17893,16 @@
           <t>40.72055787280767</t>
         </is>
       </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t>41.24982839433279</t>
+        </is>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>0.9995785650846067</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -16368,6 +18000,16 @@
           <t>38.33877389893932</t>
         </is>
       </c>
+      <c r="T164" t="inlineStr">
+        <is>
+          <t>38.987692806565846</t>
+        </is>
+      </c>
+      <c r="U164" t="inlineStr">
+        <is>
+          <t>0.9991843698269687</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -16465,6 +18107,16 @@
           <t>37.779876548598224</t>
         </is>
       </c>
+      <c r="T165" t="inlineStr">
+        <is>
+          <t>38.55917560058059</t>
+        </is>
+      </c>
+      <c r="U165" t="inlineStr">
+        <is>
+          <t>0.9991676151969889</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -16562,6 +18214,16 @@
           <t>34.90560311125649</t>
         </is>
       </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t>35.95920295225154</t>
+        </is>
+      </c>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>0.9983844355303858</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -16659,6 +18321,16 @@
           <t>34.32856888578007</t>
         </is>
       </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>35.47867513917512</t>
+        </is>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>0.9983291082093554</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -16756,6 +18428,16 @@
           <t>31.313282809776474</t>
         </is>
       </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t>32.64172586237124</t>
+        </is>
+      </c>
+      <c r="U168" t="inlineStr">
+        <is>
+          <t>0.9965508472506152</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -16853,6 +18535,16 @@
           <t>30.84932039709066</t>
         </is>
       </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t>32.23072043882687</t>
+        </is>
+      </c>
+      <c r="U169" t="inlineStr">
+        <is>
+          <t>0.9964052347495908</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -16950,6 +18642,16 @@
           <t>41.315064921991045</t>
         </is>
       </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>41.116547922141045</t>
+        </is>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>0.9994799733194023</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -17047,6 +18749,16 @@
           <t>40.59667239677214</t>
         </is>
       </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>40.68091817817532</t>
+        </is>
+      </c>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>0.9994573716269642</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -17144,6 +18856,16 @@
           <t>37.70313450795652</t>
         </is>
       </c>
+      <c r="T172" t="inlineStr">
+        <is>
+          <t>37.938654326468566</t>
+        </is>
+      </c>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>0.9988114069863654</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -17241,6 +18963,16 @@
           <t>37.00526401876999</t>
         </is>
       </c>
+      <c r="T173" t="inlineStr">
+        <is>
+          <t>37.51883538629448</t>
+        </is>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>0.998781752813069</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -17338,6 +19070,16 @@
           <t>33.98315952754679</t>
         </is>
       </c>
+      <c r="T174" t="inlineStr">
+        <is>
+          <t>34.843388742109916</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>0.9975322993995094</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -17435,6 +19177,16 @@
           <t>33.32810141866317</t>
         </is>
       </c>
+      <c r="T175" t="inlineStr">
+        <is>
+          <t>34.41702033511553</t>
+        </is>
+      </c>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>0.9974640987851835</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -17532,6 +19284,16 @@
           <t>30.57665721372961</t>
         </is>
       </c>
+      <c r="T176" t="inlineStr">
+        <is>
+          <t>31.850453764420635</t>
+        </is>
+      </c>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>0.9948468454507019</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -17629,6 +19391,16 @@
           <t>30.272439385051143</t>
         </is>
       </c>
+      <c r="T177" t="inlineStr">
+        <is>
+          <t>31.629862642313164</t>
+        </is>
+      </c>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>0.9947771621073717</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -17726,6 +19498,16 @@
           <t>42.162558542005975</t>
         </is>
       </c>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>42.53081961766975</t>
+        </is>
+      </c>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>0.9997454929339448</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -17823,6 +19605,16 @@
           <t>41.793995343062285</t>
         </is>
       </c>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>42.30066002044624</t>
+        </is>
+      </c>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>0.9997396294256138</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -17920,6 +19712,16 @@
           <t>39.974637601634846</t>
         </is>
       </c>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>40.230358514074084</t>
+        </is>
+      </c>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>0.999487577365374</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -18017,6 +19819,16 @@
           <t>39.740511602820916</t>
         </is>
       </c>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>40.08438061153865</t>
+        </is>
+      </c>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>0.9994842579162689</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -18114,6 +19926,16 @@
           <t>37.613240610011374</t>
         </is>
       </c>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>37.758998994664154</t>
+        </is>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>0.9989613092193365</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -18211,6 +20033,16 @@
           <t>37.43144660151772</t>
         </is>
       </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>37.64105032054039</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>0.9989537283412515</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -18308,6 +20140,16 @@
           <t>35.1248040488974</t>
         </is>
       </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>35.14253797845409</t>
+        </is>
+      </c>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>0.9978354655459549</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -18405,6 +20247,16 @@
           <t>35.02673157164213</t>
         </is>
       </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>35.13678286671781</t>
+        </is>
+      </c>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>0.9978699966575838</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -18502,6 +20354,16 @@
           <t>42.255608476560326</t>
         </is>
       </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>41.73888897155902</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>0.9996654858163413</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -18599,6 +20461,16 @@
           <t>41.55328222548854</t>
         </is>
       </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>41.24861968123176</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr">
+        <is>
+          <t>0.9996480521792126</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -18696,6 +20568,16 @@
           <t>38.3442074120086</t>
         </is>
       </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>38.356209992885695</t>
+        </is>
+      </c>
+      <c r="U188" t="inlineStr">
+        <is>
+          <t>0.9992383133012174</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -18793,6 +20675,16 @@
           <t>37.71660497767403</t>
         </is>
       </c>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>37.874477949288625</t>
+        </is>
+      </c>
+      <c r="U189" t="inlineStr">
+        <is>
+          <t>0.999198796432886</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -18890,6 +20782,16 @@
           <t>34.31084677696036</t>
         </is>
       </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>34.98153148990147</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>0.9983642312865975</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -18987,6 +20889,16 @@
           <t>33.78785474230306</t>
         </is>
       </c>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>34.54611909197635</t>
+        </is>
+      </c>
+      <c r="U191" t="inlineStr">
+        <is>
+          <t>0.9983169435785744</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -19084,6 +20996,16 @@
           <t>30.529163611913393</t>
         </is>
       </c>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>31.61492260322032</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>0.9965208680924545</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -19181,9 +21103,19 @@
           <t>30.10584225096775</t>
         </is>
       </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>31.232220538666354</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>0.9964479953806454</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S193"/>
+  <autoFilter ref="A1:U193"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19194,7 +21126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N97"/>
+  <dimension ref="A1:P97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19211,6 +21143,8 @@
     <col width="17" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19284,6 +21218,16 @@
           <t>psnr_hvs_m_luma_delta</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>psnr_rgb_delta</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>msssim_rgb_delta</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -19330,6 +21274,12 @@
       <c r="N2" t="n">
         <v>-0.9491950728158187</v>
       </c>
+      <c r="O2" t="n">
+        <v>-0.6546541023114898</v>
+      </c>
+      <c r="P2" t="n">
+        <v>-1.514475576525065e-05</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -19376,6 +21326,12 @@
       <c r="N3" t="n">
         <v>-0.8852457174701343</v>
       </c>
+      <c r="O3" t="n">
+        <v>-0.7000931861931932</v>
+      </c>
+      <c r="P3" t="n">
+        <v>-4.659654802574575e-05</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -19422,6 +21378,12 @@
       <c r="N4" t="n">
         <v>-0.7376030158640674</v>
       </c>
+      <c r="O4" t="n">
+        <v>-0.6727403643026051</v>
+      </c>
+      <c r="P4" t="n">
+        <v>-0.000182572936802794</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -19468,6 +21430,12 @@
       <c r="N5" t="n">
         <v>-0.4947592101989571</v>
       </c>
+      <c r="O5" t="n">
+        <v>-0.5043403107298516</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-0.0005142440885145261</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -19514,6 +21482,12 @@
       <c r="N6" t="n">
         <v>-0.6424932306992375</v>
       </c>
+      <c r="O6" t="n">
+        <v>-0.4202813597909412</v>
+      </c>
+      <c r="P6" t="n">
+        <v>-7.60604447385127e-05</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -19560,6 +21534,12 @@
       <c r="N7" t="n">
         <v>-0.4669538892147571</v>
       </c>
+      <c r="O7" t="n">
+        <v>-0.3590805282941218</v>
+      </c>
+      <c r="P7" t="n">
+        <v>-0.0001171525289078712</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -19606,6 +21586,12 @@
       <c r="N8" t="n">
         <v>-0.2951136159788987</v>
       </c>
+      <c r="O8" t="n">
+        <v>-0.218915913349278</v>
+      </c>
+      <c r="P8" t="n">
+        <v>-9.316150184490724e-05</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -19652,6 +21638,12 @@
       <c r="N9" t="n">
         <v>-0.1305070077488502</v>
       </c>
+      <c r="O9" t="n">
+        <v>-0.1397208171860669</v>
+      </c>
+      <c r="P9" t="n">
+        <v>-8.072897241551136e-05</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -19698,6 +21690,12 @@
       <c r="N10" t="n">
         <v>-0.3896092323165661</v>
       </c>
+      <c r="O10" t="n">
+        <v>-0.2511419359465989</v>
+      </c>
+      <c r="P10" t="n">
+        <v>-5.769781424969089e-06</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -19744,6 +21742,12 @@
       <c r="N11" t="n">
         <v>-0.3507811606382845</v>
       </c>
+      <c r="O11" t="n">
+        <v>-0.2492917777463504</v>
+      </c>
+      <c r="P11" t="n">
+        <v>-1.908554807994456e-05</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -19790,6 +21794,12 @@
       <c r="N12" t="n">
         <v>-0.3664389132438188</v>
       </c>
+      <c r="O12" t="n">
+        <v>-0.2641614822565543</v>
+      </c>
+      <c r="P12" t="n">
+        <v>-1.109468544102654e-05</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19836,6 +21846,12 @@
       <c r="N13" t="n">
         <v>-0.2856181335272296</v>
       </c>
+      <c r="O13" t="n">
+        <v>-0.1605976701399925</v>
+      </c>
+      <c r="P13" t="n">
+        <v>2.402663417055972e-05</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19882,6 +21898,12 @@
       <c r="N14" t="n">
         <v>-0.7174440180052741</v>
       </c>
+      <c r="O14" t="n">
+        <v>-0.4855802546308965</v>
+      </c>
+      <c r="P14" t="n">
+        <v>-2.871168722162754e-05</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -19928,6 +21950,12 @@
       <c r="N15" t="n">
         <v>-0.6772619535619384</v>
       </c>
+      <c r="O15" t="n">
+        <v>-0.4909920472460954</v>
+      </c>
+      <c r="P15" t="n">
+        <v>-5.870545966779606e-05</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -19974,6 +22002,12 @@
       <c r="N16" t="n">
         <v>-0.5355481039783498</v>
       </c>
+      <c r="O16" t="n">
+        <v>-0.4515609903788302</v>
+      </c>
+      <c r="P16" t="n">
+        <v>-0.0001242941035251022</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -20020,6 +22054,12 @@
       <c r="N17" t="n">
         <v>-0.2535139186740487</v>
       </c>
+      <c r="O17" t="n">
+        <v>-0.1953405587772039</v>
+      </c>
+      <c r="P17" t="n">
+        <v>-6.967391393863931e-05</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -20066,6 +22106,12 @@
       <c r="N18" t="n">
         <v>-0.7381030055934872</v>
       </c>
+      <c r="O18" t="n">
+        <v>-0.451903819864647</v>
+      </c>
+      <c r="P18" t="n">
+        <v>-2.152461690418939e-05</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -20112,6 +22158,12 @@
       <c r="N19" t="n">
         <v>-0.5727760681159069</v>
       </c>
+      <c r="O19" t="n">
+        <v>-0.3945119350187767</v>
+      </c>
+      <c r="P19" t="n">
+        <v>-3.275414429515511e-05</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -20158,6 +22210,12 @@
       <c r="N20" t="n">
         <v>-0.5747021600015998</v>
       </c>
+      <c r="O20" t="n">
+        <v>-0.3875053747392556</v>
+      </c>
+      <c r="P20" t="n">
+        <v>-8.186521461761576e-05</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -20204,6 +22262,12 @@
       <c r="N21" t="n">
         <v>-0.2668345372443213</v>
       </c>
+      <c r="O21" t="n">
+        <v>-0.2026216934610758</v>
+      </c>
+      <c r="P21" t="n">
+        <v>-3.932973167020126e-05</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -20250,6 +22314,12 @@
       <c r="N22" t="n">
         <v>-0.7249115147930567</v>
       </c>
+      <c r="O22" t="n">
+        <v>-0.5024411742467976</v>
+      </c>
+      <c r="P22" t="n">
+        <v>-9.341537446250214e-06</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -20296,6 +22366,12 @@
       <c r="N23" t="n">
         <v>-0.6872156257005386</v>
       </c>
+      <c r="O23" t="n">
+        <v>-0.5074931150177804</v>
+      </c>
+      <c r="P23" t="n">
+        <v>-1.498770282837292e-05</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -20342,6 +22418,12 @@
       <c r="N24" t="n">
         <v>-0.6053405934418947</v>
       </c>
+      <c r="O24" t="n">
+        <v>-0.4965791803644706</v>
+      </c>
+      <c r="P24" t="n">
+        <v>-2.007887892963023e-05</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -20388,6 +22470,12 @@
       <c r="N25" t="n">
         <v>-0.471907520067024</v>
       </c>
+      <c r="O25" t="n">
+        <v>-0.4790938562752203</v>
+      </c>
+      <c r="P25" t="n">
+        <v>-0.0001305181947860445</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -20434,6 +22522,12 @@
       <c r="N26" t="n">
         <v>-0.3114715674639399</v>
       </c>
+      <c r="O26" t="n">
+        <v>-0.2097463471433514</v>
+      </c>
+      <c r="P26" t="n">
+        <v>-9.082150699724068e-06</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -20480,6 +22574,12 @@
       <c r="N27" t="n">
         <v>-0.2859047041744276</v>
       </c>
+      <c r="O27" t="n">
+        <v>-0.2025300903431813</v>
+      </c>
+      <c r="P27" t="n">
+        <v>-1.401017251512204e-05</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -20526,6 +22626,12 @@
       <c r="N28" t="n">
         <v>-0.2453952632466638</v>
       </c>
+      <c r="O28" t="n">
+        <v>-0.1443291072859836</v>
+      </c>
+      <c r="P28" t="n">
+        <v>-6.31163174757976e-06</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -20572,6 +22678,12 @@
       <c r="N29" t="n">
         <v>-0.1686551123060624</v>
       </c>
+      <c r="O29" t="n">
+        <v>-0.05047752238021275</v>
+      </c>
+      <c r="P29" t="n">
+        <v>3.94344324525786e-05</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -20618,6 +22730,12 @@
       <c r="N30" t="n">
         <v>-1.014834788637188</v>
       </c>
+      <c r="O30" t="n">
+        <v>-0.6459578846175305</v>
+      </c>
+      <c r="P30" t="n">
+        <v>-1.317114680654541e-05</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -20664,6 +22782,12 @@
       <c r="N31" t="n">
         <v>-0.7785566545374181</v>
       </c>
+      <c r="O31" t="n">
+        <v>-0.5826051250504563</v>
+      </c>
+      <c r="P31" t="n">
+        <v>-2.956576366386354e-05</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -20710,6 +22834,12 @@
       <c r="N32" t="n">
         <v>-0.5902452709435906</v>
       </c>
+      <c r="O32" t="n">
+        <v>-0.4813491445387115</v>
+      </c>
+      <c r="P32" t="n">
+        <v>-2.820311114803964e-05</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -20756,6 +22886,12 @@
       <c r="N33" t="n">
         <v>-0.415740223942997</v>
       </c>
+      <c r="O33" t="n">
+        <v>-0.3475944726641345</v>
+      </c>
+      <c r="P33" t="n">
+        <v>-6.064009625772471e-05</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -20802,6 +22938,12 @@
       <c r="N34" t="n">
         <v>-0.3904012679301516</v>
       </c>
+      <c r="O34" t="n">
+        <v>-0.2581527456447077</v>
+      </c>
+      <c r="P34" t="n">
+        <v>-1.604959195511402e-05</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -20848,6 +22990,12 @@
       <c r="N35" t="n">
         <v>-0.2789971211823996</v>
       </c>
+      <c r="O35" t="n">
+        <v>-0.2108561071411543</v>
+      </c>
+      <c r="P35" t="n">
+        <v>-9.543964580305264e-06</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -20894,6 +23042,12 @@
       <c r="N36" t="n">
         <v>-0.3299583616241293</v>
       </c>
+      <c r="O36" t="n">
+        <v>-0.2485283792105832</v>
+      </c>
+      <c r="P36" t="n">
+        <v>-2.251499463390427e-05</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -20940,6 +23094,12 @@
       <c r="N37" t="n">
         <v>-0.2311332374532071</v>
       </c>
+      <c r="O37" t="n">
+        <v>-0.2131940929677256</v>
+      </c>
+      <c r="P37" t="n">
+        <v>-3.721964810732281e-05</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -20986,6 +23146,12 @@
       <c r="N38" t="n">
         <v>-0.4831876814571885</v>
       </c>
+      <c r="O38" t="n">
+        <v>-0.3315024326718046</v>
+      </c>
+      <c r="P38" t="n">
+        <v>-1.785161866407758e-05</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -21032,6 +23198,12 @@
       <c r="N39" t="n">
         <v>-0.2551168948275802</v>
       </c>
+      <c r="O39" t="n">
+        <v>-0.1941777740171275</v>
+      </c>
+      <c r="P39" t="n">
+        <v>-1.118282195033959e-05</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -21078,6 +23250,12 @@
       <c r="N40" t="n">
         <v>-0.1985596525988882</v>
       </c>
+      <c r="O40" t="n">
+        <v>-0.1541307158004557</v>
+      </c>
+      <c r="P40" t="n">
+        <v>-3.675260376034828e-06</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -21124,6 +23302,12 @@
       <c r="N41" t="n">
         <v>-0.1380335110060571</v>
       </c>
+      <c r="O41" t="n">
+        <v>-0.135965449859178</v>
+      </c>
+      <c r="P41" t="n">
+        <v>1.035581405206543e-05</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -21170,6 +23354,12 @@
       <c r="N42" t="n">
         <v>-0.7924273663408599</v>
       </c>
+      <c r="O42" t="n">
+        <v>-0.4823929883119291</v>
+      </c>
+      <c r="P42" t="n">
+        <v>-1.612677358686643e-05</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -21216,6 +23406,12 @@
       <c r="N43" t="n">
         <v>-0.6876474387150466</v>
       </c>
+      <c r="O43" t="n">
+        <v>-0.4825833952252196</v>
+      </c>
+      <c r="P43" t="n">
+        <v>-2.766940065046519e-05</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -21262,6 +23458,12 @@
       <c r="N44" t="n">
         <v>-0.4654936333151696</v>
       </c>
+      <c r="O44" t="n">
+        <v>-0.3579709367194042</v>
+      </c>
+      <c r="P44" t="n">
+        <v>-6.748386905119919e-05</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -21308,6 +23510,12 @@
       <c r="N45" t="n">
         <v>-0.2807734266247337</v>
       </c>
+      <c r="O45" t="n">
+        <v>-0.2759431931771985</v>
+      </c>
+      <c r="P45" t="n">
+        <v>-0.0001989958657776514</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -21354,6 +23562,12 @@
       <c r="N46" t="n">
         <v>-0.6083343530578631</v>
       </c>
+      <c r="O46" t="n">
+        <v>-0.425041091666067</v>
+      </c>
+      <c r="P46" t="n">
+        <v>-9.917423538396974e-06</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -21400,6 +23614,12 @@
       <c r="N47" t="n">
         <v>-0.4737867315204269</v>
       </c>
+      <c r="O47" t="n">
+        <v>-0.3666633309359852</v>
+      </c>
+      <c r="P47" t="n">
+        <v>-2.115424404458555e-05</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -21446,6 +23666,12 @@
       <c r="N48" t="n">
         <v>-0.3723017971066724</v>
       </c>
+      <c r="O48" t="n">
+        <v>-0.2738506958271003</v>
+      </c>
+      <c r="P48" t="n">
+        <v>-3.052171701878326e-05</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -21492,6 +23718,12 @@
       <c r="N49" t="n">
         <v>-0.2072018979382904</v>
       </c>
+      <c r="O49" t="n">
+        <v>-0.1754177271484139</v>
+      </c>
+      <c r="P49" t="n">
+        <v>-1.327887701552122e-05</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -21538,6 +23770,12 @@
       <c r="N50" t="n">
         <v>-1.147446822201893</v>
       </c>
+      <c r="O50" t="n">
+        <v>-0.6677391457441075</v>
+      </c>
+      <c r="P50" t="n">
+        <v>-1.444799619743087e-05</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -21584,6 +23822,12 @@
       <c r="N51" t="n">
         <v>-1.031977333505921</v>
       </c>
+      <c r="O51" t="n">
+        <v>-0.7278302278517543</v>
+      </c>
+      <c r="P51" t="n">
+        <v>-3.829602478866434e-05</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -21630,6 +23874,12 @@
       <c r="N52" t="n">
         <v>-0.9633709947894005</v>
       </c>
+      <c r="O52" t="n">
+        <v>-0.807296532379759</v>
+      </c>
+      <c r="P52" t="n">
+        <v>-0.0001205225436896606</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -21676,6 +23926,12 @@
       <c r="N53" t="n">
         <v>-0.6057493386547854</v>
       </c>
+      <c r="O53" t="n">
+        <v>-0.5545340192372485</v>
+      </c>
+      <c r="P53" t="n">
+        <v>-0.0001994054549432356</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -21722,6 +23978,12 @@
       <c r="N54" t="n">
         <v>-0.8606583043086715</v>
       </c>
+      <c r="O54" t="n">
+        <v>-0.5034482319646116</v>
+      </c>
+      <c r="P54" t="n">
+        <v>-1.17389070108942e-05</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -21768,6 +24030,12 @@
       <c r="N55" t="n">
         <v>-0.7528713319675902</v>
       </c>
+      <c r="O55" t="n">
+        <v>-0.5539647071413043</v>
+      </c>
+      <c r="P55" t="n">
+        <v>-5.273799728411355e-05</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -21814,6 +24082,12 @@
       <c r="N56" t="n">
         <v>-0.518211485142885</v>
       </c>
+      <c r="O56" t="n">
+        <v>-0.4101632741078944</v>
+      </c>
+      <c r="P56" t="n">
+        <v>-0.0001031352522343765</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -21860,6 +24134,12 @@
       <c r="N57" t="n">
         <v>-0.2426802800166286</v>
       </c>
+      <c r="O57" t="n">
+        <v>-0.2162621280537884</v>
+      </c>
+      <c r="P57" t="n">
+        <v>-0.0001257118226098974</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -21906,6 +24186,12 @@
       <c r="N58" t="n">
         <v>-0.8644708164471027</v>
       </c>
+      <c r="O58" t="n">
+        <v>-0.5717625855310331</v>
+      </c>
+      <c r="P58" t="n">
+        <v>-6.720960381678687e-06</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -21952,6 +24238,12 @@
       <c r="N59" t="n">
         <v>-0.7338785355891062</v>
       </c>
+      <c r="O59" t="n">
+        <v>-0.4995130197542892</v>
+      </c>
+      <c r="P59" t="n">
+        <v>-1.05063271629291e-05</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -21998,6 +24290,12 @@
       <c r="N60" t="n">
         <v>-0.4155820635773964</v>
       </c>
+      <c r="O60" t="n">
+        <v>-0.3320264014753533</v>
+      </c>
+      <c r="P60" t="n">
+        <v>-1.466860681287319e-05</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -22044,6 +24342,12 @@
       <c r="N61" t="n">
         <v>-0.2351185971113878</v>
       </c>
+      <c r="O61" t="n">
+        <v>-0.2012754156922085</v>
+      </c>
+      <c r="P61" t="n">
+        <v>-1.65383344286063e-05</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -22090,6 +24394,12 @@
       <c r="N62" t="n">
         <v>-0.6524254119115227</v>
       </c>
+      <c r="O62" t="n">
+        <v>-0.4559227021070527</v>
+      </c>
+      <c r="P62" t="n">
+        <v>-1.178570069948481e-05</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -22136,6 +24446,12 @@
       <c r="N63" t="n">
         <v>-0.6541559407807398</v>
       </c>
+      <c r="O63" t="n">
+        <v>-0.5510811651973668</v>
+      </c>
+      <c r="P63" t="n">
+        <v>-3.185306435637969e-05</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -22182,6 +24498,12 @@
       <c r="N64" t="n">
         <v>-0.5809121027143007</v>
       </c>
+      <c r="O64" t="n">
+        <v>-0.5010510968791806</v>
+      </c>
+      <c r="P64" t="n">
+        <v>-7.302485320481722e-05</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -22228,6 +24550,12 @@
       <c r="N65" t="n">
         <v>-0.349388324402014</v>
       </c>
+      <c r="O65" t="n">
+        <v>-0.3229040227412128</v>
+      </c>
+      <c r="P65" t="n">
+        <v>-0.0001175469483127856</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -22274,6 +24602,12 @@
       <c r="N66" t="n">
         <v>-0.5274192570471854</v>
       </c>
+      <c r="O66" t="n">
+        <v>-0.3630363283922264</v>
+      </c>
+      <c r="P66" t="n">
+        <v>-6.153915713458247e-06</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -22320,6 +24654,12 @@
       <c r="N67" t="n">
         <v>-0.356023127369248</v>
       </c>
+      <c r="O67" t="n">
+        <v>-0.2555716949605298</v>
+      </c>
+      <c r="P67" t="n">
+        <v>-1.154632999089689e-05</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -22366,6 +24706,12 @@
       <c r="N68" t="n">
         <v>-0.1918592275011051</v>
       </c>
+      <c r="O68" t="n">
+        <v>-0.1800704868111112</v>
+      </c>
+      <c r="P68" t="n">
+        <v>-2.851285158833594e-05</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -22412,6 +24758,12 @@
       <c r="N69" t="n">
         <v>-0.1297348346419085</v>
       </c>
+      <c r="O69" t="n">
+        <v>-0.1035446672308566</v>
+      </c>
+      <c r="P69" t="n">
+        <v>-1.099783730473813e-05</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -22458,6 +24810,12 @@
       <c r="N70" t="n">
         <v>-1.197951034593125</v>
       </c>
+      <c r="O70" t="n">
+        <v>-0.7185935680678028</v>
+      </c>
+      <c r="P70" t="n">
+        <v>-5.514667501405057e-05</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -22504,6 +24862,12 @@
       <c r="N71" t="n">
         <v>-0.7403279477573008</v>
       </c>
+      <c r="O71" t="n">
+        <v>-0.5272062360678547</v>
+      </c>
+      <c r="P71" t="n">
+        <v>-0.0001087145790545918</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -22550,6 +24914,12 @@
       <c r="N72" t="n">
         <v>-0.6189262897934853</v>
       </c>
+      <c r="O72" t="n">
+        <v>-0.4580565383461987</v>
+      </c>
+      <c r="P72" t="n">
+        <v>-0.0001830505171133145</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -22596,6 +24966,12 @@
       <c r="N73" t="n">
         <v>-0.4740176443822079</v>
       </c>
+      <c r="O73" t="n">
+        <v>-0.39639404171999</v>
+      </c>
+      <c r="P73" t="n">
+        <v>-0.0003162936674262484</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -22642,6 +25018,12 @@
       <c r="N74" t="n">
         <v>-0.6085139684214553</v>
       </c>
+      <c r="O74" t="n">
+        <v>-0.4266587525194865</v>
+      </c>
+      <c r="P74" t="n">
+        <v>-9.391810170900072e-06</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -22688,6 +25070,12 @@
       <c r="N75" t="n">
         <v>-0.7530114373428418</v>
       </c>
+      <c r="O75" t="n">
+        <v>-0.5798135140690874</v>
+      </c>
+      <c r="P75" t="n">
+        <v>-3.476799222101867e-05</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -22734,6 +25122,12 @@
       <c r="N76" t="n">
         <v>-0.7431300509284355</v>
       </c>
+      <c r="O76" t="n">
+        <v>-0.5721508767634162</v>
+      </c>
+      <c r="P76" t="n">
+        <v>-6.115527217853689e-05</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -22780,6 +25174,12 @@
       <c r="N77" t="n">
         <v>-0.252898078328144</v>
       </c>
+      <c r="O77" t="n">
+        <v>-0.2340601168775009</v>
+      </c>
+      <c r="P77" t="n">
+        <v>-6.702217911458419e-05</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -22826,6 +25226,12 @@
       <c r="N78" t="n">
         <v>-0.5492103466828837</v>
       </c>
+      <c r="O78" t="n">
+        <v>-0.3130492757951302</v>
+      </c>
+      <c r="P78" t="n">
+        <v>-1.155574412825544e-06</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -22872,6 +25278,12 @@
       <c r="N79" t="n">
         <v>-0.6383053726008896</v>
       </c>
+      <c r="O79" t="n">
+        <v>-0.3906871128275426</v>
+      </c>
+      <c r="P79" t="n">
+        <v>-2.880307746311317e-06</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -22918,6 +25330,12 @@
       <c r="N80" t="n">
         <v>-0.6889687457984834</v>
       </c>
+      <c r="O80" t="n">
+        <v>-0.5080782273851412</v>
+      </c>
+      <c r="P80" t="n">
+        <v>-1.313714785744491e-05</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -22964,6 +25382,12 @@
       <c r="N81" t="n">
         <v>-0.2396625959096852</v>
       </c>
+      <c r="O81" t="n">
+        <v>-0.1696269009649072</v>
+      </c>
+      <c r="P81" t="n">
+        <v>-6.499047538688352e-06</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -23010,6 +25434,12 @@
       <c r="N82" t="n">
         <v>-0.5750359442745605</v>
       </c>
+      <c r="O82" t="n">
+        <v>-0.4013807675101688</v>
+      </c>
+      <c r="P82" t="n">
+        <v>-1.023458442361846e-05</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -23056,6 +25486,12 @@
       <c r="N83" t="n">
         <v>-0.5588973503410983</v>
       </c>
+      <c r="O83" t="n">
+        <v>-0.4285172059852584</v>
+      </c>
+      <c r="P83" t="n">
+        <v>-1.675462997974275e-05</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -23102,6 +25538,12 @@
       <c r="N84" t="n">
         <v>-0.5770342254764174</v>
       </c>
+      <c r="O84" t="n">
+        <v>-0.4805278130764208</v>
+      </c>
+      <c r="P84" t="n">
+        <v>-5.532732103041837e-05</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -23148,6 +25590,12 @@
       <c r="N85" t="n">
         <v>-0.4639624126858131</v>
       </c>
+      <c r="O85" t="n">
+        <v>-0.411005423544367</v>
+      </c>
+      <c r="P85" t="n">
+        <v>-0.0001456125010244058</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -23194,6 +25642,12 @@
       <c r="N86" t="n">
         <v>-0.7183925252189027</v>
       </c>
+      <c r="O86" t="n">
+        <v>-0.4356297439657268</v>
+      </c>
+      <c r="P86" t="n">
+        <v>-2.260169243806232e-05</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -23240,6 +25694,12 @@
       <c r="N87" t="n">
         <v>-0.6978704891865277</v>
       </c>
+      <c r="O87" t="n">
+        <v>-0.4198189401740891</v>
+      </c>
+      <c r="P87" t="n">
+        <v>-2.965417329636733e-05</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -23286,6 +25746,12 @@
       <c r="N88" t="n">
         <v>-0.6550581088836225</v>
       </c>
+      <c r="O88" t="n">
+        <v>-0.4263684069943849</v>
+      </c>
+      <c r="P88" t="n">
+        <v>-6.82006143258862e-05</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -23332,6 +25798,12 @@
       <c r="N89" t="n">
         <v>-0.3042178286784676</v>
       </c>
+      <c r="O89" t="n">
+        <v>-0.2205911221074714</v>
+      </c>
+      <c r="P89" t="n">
+        <v>-6.968334333024018e-05</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -23378,6 +25850,12 @@
       <c r="N90" t="n">
         <v>-0.3685631989436899</v>
       </c>
+      <c r="O90" t="n">
+        <v>-0.230159597223512</v>
+      </c>
+      <c r="P90" t="n">
+        <v>-5.863508330983258e-06</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -23424,6 +25902,12 @@
       <c r="N91" t="n">
         <v>-0.2341259988139299</v>
       </c>
+      <c r="O91" t="n">
+        <v>-0.1459779025354351</v>
+      </c>
+      <c r="P91" t="n">
+        <v>-3.319449105032568e-06</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -23470,6 +25954,12 @@
       <c r="N92" t="n">
         <v>-0.1817940084936538</v>
       </c>
+      <c r="O92" t="n">
+        <v>-0.1179486741237668</v>
+      </c>
+      <c r="P92" t="n">
+        <v>-7.58087808494512e-06</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -23516,6 +26006,12 @@
       <c r="N93" t="n">
         <v>-0.09807247725527191</v>
       </c>
+      <c r="O93" t="n">
+        <v>-0.00575511173627774</v>
+      </c>
+      <c r="P93" t="n">
+        <v>3.453111162887712e-05</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -23562,6 +26058,12 @@
       <c r="N94" t="n">
         <v>-0.7023262510717885</v>
       </c>
+      <c r="O94" t="n">
+        <v>-0.4902692903272623</v>
+      </c>
+      <c r="P94" t="n">
+        <v>-1.743363712869428e-05</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -23608,6 +26110,12 @@
       <c r="N95" t="n">
         <v>-0.6276024343345696</v>
       </c>
+      <c r="O95" t="n">
+        <v>-0.48173204359707</v>
+      </c>
+      <c r="P95" t="n">
+        <v>-3.951686833136847e-05</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -23654,6 +26162,12 @@
       <c r="N96" t="n">
         <v>-0.5229920346572996</v>
       </c>
+      <c r="O96" t="n">
+        <v>-0.4354123979251199</v>
+      </c>
+      <c r="P96" t="n">
+        <v>-4.728770802309157e-05</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -23700,9 +26214,15 @@
       <c r="N97" t="n">
         <v>-0.4233213609456428</v>
       </c>
+      <c r="O97" t="n">
+        <v>-0.3827020645539676</v>
+      </c>
+      <c r="P97" t="n">
+        <v>-7.287271180911326e-05</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N97"/>
+  <autoFilter ref="A1:P97"/>
   <conditionalFormatting sqref="E2:E97">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -23783,6 +26303,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="O2:O97">
+    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="22" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P2:P97">
+    <cfRule type="cellIs" priority="23" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="24" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23793,7 +26329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24072,9 +26608,65 @@
         <v>-0.3127394616214333</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>psnr_rgb</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>24</v>
+      </c>
+      <c r="C10" t="n">
+        <v>7.091271231023569</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3.967536188438414</v>
+      </c>
+      <c r="E10" t="n">
+        <v>9.679231487277185</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.368146420094105</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0.6072957154009749</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-0.2513305963505965</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>msssim_rgb</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>24</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2.407472213563013</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-0.1772565834730955</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4.92180866543217</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-4.93463993038291e-05</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-0.0001825742912845522</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8.408051438964316e-07</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H9"/>
-  <conditionalFormatting sqref="C2:C9">
+  <autoFilter ref="A1:H11"/>
+  <conditionalFormatting sqref="C2:C11">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -24082,7 +26674,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D9">
+  <conditionalFormatting sqref="D2:D11">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -24090,7 +26682,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E9">
+  <conditionalFormatting sqref="E2:E11">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -24098,7 +26690,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F9">
+  <conditionalFormatting sqref="F2:F11">
     <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -24106,7 +26698,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G9">
+  <conditionalFormatting sqref="G2:G11">
     <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -24114,7 +26706,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H9">
+  <conditionalFormatting sqref="H2:H11">
     <cfRule type="cellIs" priority="11" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>